<commit_message>
Refinando filtros de busca
</commit_message>
<xml_diff>
--- a/data/alertas.xlsx
+++ b/data/alertas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1058,6 +1058,40 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46308.83702546296</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pore Refiner Creamy Skincare 70 Pads com Ácido Salicílico</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>132.04</v>
+      </c>
+      <c r="D20" t="n">
+        <v>140</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>🐾 BOTE CERTEIRO! Pore Refiner Creamy Skincare 70 Pads com Ácido Salicílico caiu 0,0% e está em R$ 132,04. Pode me agradecer com sachê.
+🛍️ Pore Refiner Creamy Skincare 70 Pads com Ácido Salicílico
+💰 Preço atual: R$ 132,04
+🎯 Meta: R$ 140,00
+📉 Variação: ▲ 0,0% desde a última espiada
+🔗 Ver a presa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>